<commit_message>
docs: adiciona planilha de plano e casos de teste
</commit_message>
<xml_diff>
--- a/docs/plano-e-casos-de-teste.xlsx
+++ b/docs/plano-e-casos-de-teste.xlsx
@@ -98,7 +98,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -120,11 +120,55 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -184,6 +228,8 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -573,11 +619,11 @@
           <t>INFORMAÇÕES GERAIS</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
+      <c r="B3" s="21" t="n"/>
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="22" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -590,10 +636,10 @@
           <t>Desafio QA Jr — PortData</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="22" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -606,10 +652,10 @@
           <t>GitHub (https://github.com)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="22" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -622,10 +668,10 @@
           <t>Cypress v14+ | K6 v2+ | Node.js v24+</t>
         </is>
       </c>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="22" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -638,10 +684,10 @@
           <t>Chrome</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-      <c r="F7" s="3" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -654,10 +700,10 @@
           <t>Pedro Alcântara</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n"/>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
+      <c r="C8" s="21" t="n"/>
+      <c r="D8" s="21" t="n"/>
+      <c r="E8" s="21" t="n"/>
+      <c r="F8" s="22" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -670,10 +716,10 @@
           <t>Maio/2026</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
+      <c r="C9" s="21" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="22" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -681,11 +727,11 @@
           <t>ESCOPO</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="21" t="n"/>
+      <c r="D11" s="21" t="n"/>
+      <c r="E11" s="21" t="n"/>
+      <c r="F11" s="22" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -698,10 +744,10 @@
           <t>Fluxo de autenticação (login e logout)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -714,10 +760,10 @@
           <t>Navegação entre abas e repositórios</t>
         </is>
       </c>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="22" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
@@ -730,10 +776,10 @@
           <t>Criação de repositório com XPath</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="22" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -746,10 +792,10 @@
           <t>Performance das requisições nos fluxos principais</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="22" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -762,10 +808,10 @@
           <t>Testes de segurança e acessibilidade</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="22" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -778,10 +824,10 @@
           <t>Cadastro de novo usuário</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="22" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -794,10 +840,10 @@
           <t>Funcionalidades de organização e enterprise</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="22" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
@@ -805,11 +851,11 @@
           <t>ESTRATÉGIA DE TESTES</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="21" t="n"/>
+      <c r="F20" s="22" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -827,9 +873,9 @@
           <t>Objetivo</t>
         </is>
       </c>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="21" t="n"/>
+      <c r="F21" s="22" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
@@ -847,9 +893,9 @@
           <t>Validar os fluxos funcionais completos simulando o comportamento do usuário real no browser</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="22" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
@@ -867,9 +913,9 @@
           <t>Medir o tempo de resposta das requisições HTTP nos fluxos principais e validar SLA de 3 segundos</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="22" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
@@ -877,9 +923,11 @@
           <t>RISCOS E MITIGAÇÕES</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="21" t="n"/>
+      <c r="D25" s="21" t="n"/>
+      <c r="E25" s="21" t="n"/>
+      <c r="F25" s="22" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -1044,13 +1092,13 @@
           <t>CASOS DE TESTE — Desafio QA Jr | PortData</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="21" t="n"/>
+      <c r="H1" s="22" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1366,7 +1414,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Usuário autenticado. GITHUB_REPO_NAME definido no .env</t>
+          <t>Usuário autenticado. Nome do repositório gerado dinamicamente com timestamp (Date.now()) para evitar conflitos</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -1423,7 +1471,7 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Usuário deslogado e redirecionado para a página inicial</t>
+          <t>Usuário deslogado. URL redireciona para /logout (página de confirmação) e após confirmação retorna para github.com/</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -1460,8 +1508,9 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>1. GET /login
-2. POST /session com credenciais</t>
+          <t>1. GET /login (captura authenticity_token)
+2. POST /session com e-mail, senha e token
+3. Medir tempo de resposta</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1503,7 +1552,8 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>1. GET /{username}?tab=repositories</t>
+          <t>1. GET /{username}?tab=repositories com cookie jar da sessão
+2. Medir tempo de resposta</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1545,7 +1595,8 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>1. GET /logout</t>
+          <t>1. GET /logout com cookie jar da sessão
+2. Medir tempo de resposta</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1601,12 +1652,12 @@
           <t>RESUMO DE EXECUÇÃO — Desafio QA Jr | PortData</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
+      <c r="B1" s="21" t="n"/>
+      <c r="C1" s="21" t="n"/>
+      <c r="D1" s="21" t="n"/>
+      <c r="E1" s="21" t="n"/>
+      <c r="F1" s="21" t="n"/>
+      <c r="G1" s="22" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1941,7 +1992,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Tempo médio: ~300ms</t>
+          <t>Tempo médio: 476ms | Min: 275ms | Max: 720ms | 100% checks passou</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -1978,7 +2029,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Tempo médio: ~250ms</t>
+          <t>Tempo médio: 476ms | Min: 275ms | Max: 720ms | 100% checks passou</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -2015,7 +2066,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Tempo médio: ~200ms</t>
+          <t>Tempo médio: 476ms | Min: 275ms | Max: 720ms | 100% checks passou</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -2039,9 +2090,9 @@
           <t>TOTAIS</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="22" t="n"/>
       <c r="E15" s="6">
         <f>COUNTIF(E3:E14,"✅ Passou")</f>
         <v/>

</xml_diff>

<commit_message>
docs: atualiza planilha de plano e casos de teste
</commit_message>
<xml_diff>
--- a/docs/plano-e-casos-de-teste.xlsx
+++ b/docs/plano-e-casos-de-teste.xlsx
@@ -1992,7 +1992,7 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Tempo médio: 476ms | Min: 275ms | Max: 720ms | 100% checks passou</t>
+          <t>K6 retorna métrica consolidada de todas as requisições. Avg geral: 476ms | Min: 275ms | Max: 720ms | Todos dentro do SLA de 3000ms</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Tempo médio: 476ms | Min: 275ms | Max: 720ms | 100% checks passou</t>
+          <t>K6 retorna métrica consolidada de todas as requisições. Avg geral: 476ms | Min: 275ms | Max: 720ms | Todos dentro do SLA de 3000ms</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Tempo médio: 476ms | Min: 275ms | Max: 720ms | 100% checks passou</t>
+          <t>K6 retorna métrica consolidada de todas as requisições. Avg geral: 476ms | Min: 275ms | Max: 720ms | Todos dentro do SLA de 3000ms</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">

</xml_diff>

<commit_message>
docs: organiza documentação técnica do projeto
</commit_message>
<xml_diff>
--- a/docs/plano-e-casos-de-teste.xlsx
+++ b/docs/plano-e-casos-de-teste.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30720" windowHeight="13320" activeTab="2"/>
+    <workbookView windowWidth="30720" windowHeight="13320"/>
   </bookViews>
   <sheets>
     <sheet name="Plano de Testes" sheetId="1" r:id="rId1"/>
@@ -432,7 +432,7 @@
     <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -464,6 +464,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -624,7 +631,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -687,12 +694,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -700,12 +701,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1008,79 +1003,85 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1089,10 +1090,10 @@
     <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1101,10 +1102,10 @@
     <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1113,10 +1114,10 @@
     <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1125,10 +1126,10 @@
     <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1137,23 +1138,17 @@
     <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1209,10 +1204,11 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1561,8 +1557,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1571,12 +1567,13 @@
     <col min="5" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="35" customHeight="1" spans="1:6">
+    <row r="1" ht="35" customHeight="1" spans="1:7">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:6">
+      <c r="G1" s="21"/>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:7">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -1586,7 +1583,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" ht="18" customHeight="1" spans="1:6">
+    <row r="4" ht="18" customHeight="1" spans="1:7">
       <c r="A4" s="17" t="s">
         <v>2</v>
       </c>
@@ -1598,7 +1595,7 @@
       <c r="E4" s="2"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" ht="18" customHeight="1" spans="1:6">
+    <row r="5" ht="18" customHeight="1" spans="1:7">
       <c r="A5" s="17" t="s">
         <v>4</v>
       </c>
@@ -1610,7 +1607,7 @@
       <c r="E5" s="2"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" ht="18" customHeight="1" spans="1:6">
+    <row r="6" ht="18" customHeight="1" spans="1:7">
       <c r="A6" s="17" t="s">
         <v>6</v>
       </c>
@@ -1622,7 +1619,7 @@
       <c r="E6" s="2"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" ht="18" customHeight="1" spans="1:6">
+    <row r="7" ht="18" customHeight="1" spans="1:7">
       <c r="A7" s="17" t="s">
         <v>8</v>
       </c>
@@ -1634,7 +1631,7 @@
       <c r="E7" s="2"/>
       <c r="F7" s="3"/>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:6">
+    <row r="8" ht="18" customHeight="1" spans="1:7">
       <c r="A8" s="17" t="s">
         <v>10</v>
       </c>
@@ -1646,7 +1643,7 @@
       <c r="E8" s="2"/>
       <c r="F8" s="3"/>
     </row>
-    <row r="9" ht="18" customHeight="1" spans="1:6">
+    <row r="9" ht="18" customHeight="1" spans="1:7">
       <c r="A9" s="17" t="s">
         <v>12</v>
       </c>
@@ -1658,7 +1655,7 @@
       <c r="E9" s="2"/>
       <c r="F9" s="3"/>
     </row>
-    <row r="11" ht="22" customHeight="1" spans="1:6">
+    <row r="11" ht="22" customHeight="1" spans="1:7">
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
@@ -1668,11 +1665,11 @@
       <c r="E11" s="2"/>
       <c r="F11" s="3"/>
     </row>
-    <row r="12" ht="18" customHeight="1" spans="1:6">
+    <row r="12" ht="18" customHeight="1" spans="1:7">
       <c r="A12" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="22" t="s">
         <v>16</v>
       </c>
       <c r="C12" s="2"/>
@@ -1680,11 +1677,11 @@
       <c r="E12" s="2"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" ht="18" customHeight="1" spans="1:6">
+    <row r="13" ht="18" customHeight="1" spans="1:7">
       <c r="A13" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="2"/>
@@ -1692,11 +1689,11 @@
       <c r="E13" s="2"/>
       <c r="F13" s="3"/>
     </row>
-    <row r="14" ht="18" customHeight="1" spans="1:6">
+    <row r="14" ht="18" customHeight="1" spans="1:7">
       <c r="A14" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="22" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="2"/>
@@ -1704,11 +1701,11 @@
       <c r="E14" s="2"/>
       <c r="F14" s="3"/>
     </row>
-    <row r="15" ht="18" customHeight="1" spans="1:6">
+    <row r="15" ht="18" customHeight="1" spans="1:7">
       <c r="A15" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="22" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="2"/>
@@ -1716,7 +1713,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="3"/>
     </row>
-    <row r="16" ht="18" customHeight="1" spans="1:6">
+    <row r="16" ht="18" customHeight="1" spans="1:7">
       <c r="A16" s="10" t="s">
         <v>20</v>
       </c>
@@ -1763,13 +1760,13 @@
       <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="23" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="2"/>
@@ -1815,16 +1812,16 @@
       <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D26" s="23" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2515,7 +2512,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" spans="1:7">
+    <row r="12" ht="60" customHeight="1" spans="1:7">
       <c r="A12" s="10" t="s">
         <v>106</v>
       </c>
@@ -2538,7 +2535,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1" spans="1:7">
+    <row r="13" ht="70" customHeight="1" spans="1:7">
       <c r="A13" s="5" t="s">
         <v>110</v>
       </c>

</xml_diff>